<commit_message>
Update output of fanins
</commit_message>
<xml_diff>
--- a/Usage/Output/optimize_FanIn.xlsx
+++ b/Usage/Output/optimize_FanIn.xlsx
@@ -668,10 +668,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>28480</v>
+        <v>28455</v>
       </c>
       <c r="D10" t="n">
-        <v>28480</v>
+        <v>28455</v>
       </c>
       <c r="E10" t="n">
         <v>4</v>
@@ -772,7 +772,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>15297</v>
+        <v>15253</v>
       </c>
       <c r="D14" t="n">
         <v>609</v>
@@ -1032,10 +1032,10 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>8738</v>
+        <v>8655</v>
       </c>
       <c r="D24" t="n">
-        <v>8738</v>
+        <v>8655</v>
       </c>
       <c r="E24" t="n">
         <v>69</v>
@@ -1075,7 +1075,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>scipy.optimize._optimize._minimize_newtoncg</t>
+          <t>scipy.optimize._linprog_ip._sym_solve</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1084,24 +1084,24 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>7934</v>
+        <v>7876</v>
       </c>
       <c r="D26" t="n">
-        <v>175</v>
+        <v>4040</v>
       </c>
       <c r="E26" t="n">
-        <v>192</v>
+        <v>18</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>/Users/muyeedahmed/Desktop/Gitcode/ForkedLibrary/scipy/scipy/optimize/_optimize.py</t>
+          <t>/Users/muyeedahmed/Desktop/Gitcode/ForkedLibrary/scipy/scipy/optimize/_linprog_ip.py</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>scipy.optimize._linprog_ip._sym_solve</t>
+          <t>scipy.optimize._optimize._minimize_newtoncg</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1110,17 +1110,17 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>7876</v>
+        <v>7758</v>
       </c>
       <c r="D27" t="n">
-        <v>4040</v>
+        <v>175</v>
       </c>
       <c r="E27" t="n">
-        <v>18</v>
+        <v>192</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>/Users/muyeedahmed/Desktop/Gitcode/ForkedLibrary/scipy/scipy/optimize/_linprog_ip.py</t>
+          <t>/Users/muyeedahmed/Desktop/Gitcode/ForkedLibrary/scipy/scipy/optimize/_optimize.py</t>
         </is>
       </c>
     </row>
@@ -1188,10 +1188,10 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>6104</v>
+        <v>6042</v>
       </c>
       <c r="D30" t="n">
-        <v>3566</v>
+        <v>3535</v>
       </c>
       <c r="E30" t="n">
         <v>16</v>
@@ -1396,10 +1396,10 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>3648</v>
+        <v>3617</v>
       </c>
       <c r="D38" t="n">
-        <v>3648</v>
+        <v>3617</v>
       </c>
       <c r="E38" t="n">
         <v>9</v>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2813</v>
+        <v>2776</v>
       </c>
       <c r="D42" t="n">
         <v>546</v>
@@ -1552,10 +1552,10 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2663</v>
+        <v>2675</v>
       </c>
       <c r="D44" t="n">
-        <v>2663</v>
+        <v>2675</v>
       </c>
       <c r="E44" t="n">
         <v>5</v>
@@ -2020,10 +2020,10 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>999</v>
+        <v>1005</v>
       </c>
       <c r="D62" t="n">
-        <v>999</v>
+        <v>1005</v>
       </c>
       <c r="E62" t="n">
         <v>32</v>
@@ -2410,10 +2410,10 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="D77" t="n">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="E77" t="n">
         <v>149</v>

</xml_diff>